<commit_message>
Pagina de pagamento adicionada
</commit_message>
<xml_diff>
--- a/dataset/bd_cobranca.xlsx
+++ b/dataset/bd_cobranca.xlsx
@@ -19,7 +19,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="R$ #,##0.00"/>
   </numFmts>
-  <fonts count="11">
+  <fonts count="6">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -46,32 +46,6 @@
     </font>
     <font>
       <name val="Calibri"/>
-      <sz val="9"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <b val="1"/>
-      <color rgb="001D9E75"/>
-      <sz val="9"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <b val="1"/>
-      <color rgb="00FFFFFF"/>
-      <sz val="9"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <b val="1"/>
-      <sz val="9"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <color rgb="001A1530"/>
-      <sz val="9"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
       <b val="1"/>
       <color rgb="00FFFFFF"/>
       <sz val="11"/>
@@ -83,7 +57,7 @@
       <sz val="8"/>
     </font>
   </fonts>
-  <fills count="8">
+  <fills count="5">
     <fill>
       <patternFill/>
     </fill>
@@ -102,26 +76,11 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FFFFFF"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="001D9E75"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00EDE8FF"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor rgb="00C0392B"/>
       </patternFill>
     </fill>
   </fills>
-  <borders count="4">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -145,20 +104,6 @@
     </border>
     <border>
       <left style="thin">
-        <color rgb="00C8C0F0"/>
-      </left>
-      <right style="thin">
-        <color rgb="00C8C0F0"/>
-      </right>
-      <top style="thin">
-        <color rgb="00C8C0F0"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="00C8C0F0"/>
-      </bottom>
-    </border>
-    <border>
-      <left style="thin">
         <color rgb="00C0392B"/>
       </left>
       <right style="thin">
@@ -175,7 +120,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -186,46 +131,13 @@
     <xf numFmtId="0" fontId="3" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="5" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="164" fontId="8" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="6" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="6" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="6" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="6" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="164" fontId="8" fillId="6" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="7" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="9" fillId="7" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="4" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -593,22 +505,23 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M11"/>
+  <dimension ref="A1:N7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="16" customWidth="1" min="1" max="1"/>
     <col width="14" customWidth="1" min="2" max="2"/>
     <col width="14" customWidth="1" min="3" max="3"/>
-    <col width="22" customWidth="1" min="4" max="4"/>
-    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="22" customWidth="1" min="5" max="5"/>
     <col width="16" customWidth="1" min="6" max="6"/>
     <col width="16" customWidth="1" min="7" max="7"/>
-    <col width="34" customWidth="1" min="8" max="8"/>
-    <col width="12" customWidth="1" min="9" max="9"/>
-    <col width="26" customWidth="1" min="10" max="10"/>
-    <col width="14" customWidth="1" min="11" max="11"/>
-    <col width="16" customWidth="1" min="12" max="12"/>
-    <col width="20" customWidth="1" min="13" max="13"/>
+    <col width="16" customWidth="1" min="8" max="8"/>
+    <col width="34" customWidth="1" min="9" max="9"/>
+    <col width="12" customWidth="1" min="10" max="10"/>
+    <col width="26" customWidth="1" min="11" max="11"/>
+    <col width="14" customWidth="1" min="12" max="12"/>
+    <col width="16" customWidth="1" min="13" max="13"/>
+    <col width="20" customWidth="1" min="14" max="14"/>
   </cols>
   <sheetData>
     <row r="1" ht="34" customHeight="1">
@@ -621,7 +534,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Gerado em: 22/06/2026  ·  Total de registros: 4</t>
+          <t>Gerado em: 23/06/2026  ·  Total de registros: 0</t>
         </is>
       </c>
     </row>
@@ -629,310 +542,87 @@
     <row r="4" ht="26" customHeight="1">
       <c r="A4" s="3" t="inlineStr">
         <is>
+          <t>Código</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
           <t>Data Cobrança</t>
         </is>
       </c>
-      <c r="B4" s="3" t="inlineStr">
+      <c r="C4" s="3" t="inlineStr">
         <is>
           <t>Data Vencimento</t>
         </is>
       </c>
-      <c r="C4" s="3" t="inlineStr">
+      <c r="D4" s="3" t="inlineStr">
         <is>
           <t>Data Pagamento</t>
         </is>
       </c>
-      <c r="D4" s="3" t="inlineStr">
+      <c r="E4" s="3" t="inlineStr">
         <is>
           <t>CNPJ</t>
         </is>
       </c>
-      <c r="E4" s="3" t="inlineStr">
+      <c r="F4" s="3" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
       </c>
-      <c r="F4" s="3" t="inlineStr">
+      <c r="G4" s="3" t="inlineStr">
         <is>
           <t>OM</t>
         </is>
       </c>
-      <c r="G4" s="3" t="inlineStr">
+      <c r="H4" s="3" t="inlineStr">
         <is>
           <t>Data Produção</t>
         </is>
       </c>
-      <c r="H4" s="3" t="inlineStr">
+      <c r="I4" s="3" t="inlineStr">
         <is>
           <t>Fornecedor</t>
         </is>
       </c>
-      <c r="I4" s="3" t="inlineStr">
+      <c r="J4" s="3" t="inlineStr">
         <is>
           <t>Qtd</t>
         </is>
       </c>
-      <c r="J4" s="3" t="inlineStr">
+      <c r="K4" s="3" t="inlineStr">
         <is>
           <t>Remonte / Defeito</t>
         </is>
       </c>
-      <c r="K4" s="3" t="inlineStr">
+      <c r="L4" s="3" t="inlineStr">
         <is>
           <t>Real Cortado</t>
         </is>
       </c>
-      <c r="L4" s="3" t="inlineStr">
+      <c r="M4" s="3" t="inlineStr">
         <is>
           <t>Min. Gerados</t>
         </is>
       </c>
-      <c r="M4" s="3" t="inlineStr">
+      <c r="N4" s="3" t="inlineStr">
         <is>
           <t>Valor (R$)</t>
         </is>
       </c>
     </row>
-    <row r="5" ht="17" customHeight="1">
+    <row r="5" ht="22" customHeight="1">
       <c r="A5" s="4" t="inlineStr">
         <is>
-          <t>12/06/2026</t>
-        </is>
-      </c>
-      <c r="B5" s="4" t="inlineStr">
-        <is>
-          <t>02/07/2026</t>
-        </is>
-      </c>
-      <c r="C5" s="5" t="inlineStr">
-        <is>
-          <t>19/06/2026</t>
-        </is>
-      </c>
-      <c r="D5" s="5" t="inlineStr">
-        <is>
-          <t>62.470.324/0001-40</t>
-        </is>
-      </c>
-      <c r="E5" s="6" t="inlineStr">
-        <is>
-          <t>Pago</t>
-        </is>
-      </c>
-      <c r="F5" s="7" t="n">
-        <v>300258637</v>
-      </c>
-      <c r="G5" s="4" t="inlineStr">
-        <is>
-          <t>02/06/2026</t>
-        </is>
-      </c>
-      <c r="H5" s="8" t="inlineStr">
-        <is>
-          <t>M K INDUSTRIA TEXTIL LTDA</t>
-        </is>
-      </c>
-      <c r="I5" s="4" t="n">
-        <v>71</v>
-      </c>
-      <c r="J5" s="8" t="inlineStr">
-        <is>
-          <t>ESGARÇANDO</t>
-        </is>
-      </c>
-      <c r="K5" s="4" t="n">
-        <v>798</v>
-      </c>
-      <c r="L5" s="4" t="n">
-        <v>201.64</v>
-      </c>
-      <c r="M5" s="9" t="n">
-        <v>235.9188</v>
+          <t>TOTAL HISTÓRICO</t>
+        </is>
+      </c>
+      <c r="N5" s="5" t="n">
+        <v>0</v>
       </c>
     </row>
-    <row r="6" ht="17" customHeight="1">
-      <c r="A6" s="10" t="inlineStr">
-        <is>
-          <t>12/06/2026</t>
-        </is>
-      </c>
-      <c r="B6" s="10" t="inlineStr">
-        <is>
-          <t>02/07/2026</t>
-        </is>
-      </c>
-      <c r="C6" s="11" t="inlineStr">
-        <is>
-          <t>19/06/2026</t>
-        </is>
-      </c>
-      <c r="D6" s="11" t="inlineStr">
-        <is>
-          <t>62.470.324/0001-40</t>
-        </is>
-      </c>
-      <c r="E6" s="6" t="inlineStr">
-        <is>
-          <t>Pago</t>
-        </is>
-      </c>
-      <c r="F6" s="12" t="n">
-        <v>300258637</v>
-      </c>
-      <c r="G6" s="10" t="inlineStr">
-        <is>
-          <t>02/06/2026</t>
-        </is>
-      </c>
-      <c r="H6" s="13" t="inlineStr">
-        <is>
-          <t>M K INDUSTRIA TEXTIL LTDA</t>
-        </is>
-      </c>
-      <c r="I6" s="10" t="n">
-        <v>37</v>
-      </c>
-      <c r="J6" s="13" t="inlineStr">
-        <is>
-          <t>PONTO ESTOURADO</t>
-        </is>
-      </c>
-      <c r="K6" s="10" t="n">
-        <v>798</v>
-      </c>
-      <c r="L6" s="10" t="n">
-        <v>11.47</v>
-      </c>
-      <c r="M6" s="14" t="n">
-        <v>13.4199</v>
-      </c>
-    </row>
-    <row r="7" ht="17" customHeight="1">
-      <c r="A7" s="4" t="inlineStr">
-        <is>
-          <t>12/06/2026</t>
-        </is>
-      </c>
-      <c r="B7" s="4" t="inlineStr">
-        <is>
-          <t>02/07/2026</t>
-        </is>
-      </c>
-      <c r="C7" s="5" t="inlineStr">
-        <is>
-          <t>19/06/2026</t>
-        </is>
-      </c>
-      <c r="D7" s="5" t="inlineStr">
-        <is>
-          <t>62.470.324/0001-40</t>
-        </is>
-      </c>
-      <c r="E7" s="6" t="inlineStr">
-        <is>
-          <t>Pago</t>
-        </is>
-      </c>
-      <c r="F7" s="7" t="n">
-        <v>300258637</v>
-      </c>
-      <c r="G7" s="4" t="inlineStr">
-        <is>
-          <t>02/06/2026</t>
-        </is>
-      </c>
-      <c r="H7" s="8" t="inlineStr">
-        <is>
-          <t>M K INDUSTRIA TEXTIL LTDA</t>
-        </is>
-      </c>
-      <c r="I7" s="4" t="n">
-        <v>7</v>
-      </c>
-      <c r="J7" s="8" t="inlineStr">
-        <is>
-          <t>SEM ARREMATE</t>
-        </is>
-      </c>
-      <c r="K7" s="4" t="n">
-        <v>798</v>
-      </c>
-      <c r="L7" s="4" t="n">
-        <v>2.31</v>
-      </c>
-      <c r="M7" s="9" t="n">
-        <v>2.7027</v>
-      </c>
-    </row>
-    <row r="8" ht="17" customHeight="1">
-      <c r="A8" s="10" t="inlineStr">
-        <is>
-          <t>12/06/2026</t>
-        </is>
-      </c>
-      <c r="B8" s="10" t="inlineStr">
-        <is>
-          <t>02/07/2026</t>
-        </is>
-      </c>
-      <c r="C8" s="11" t="inlineStr">
-        <is>
-          <t>19/06/2026</t>
-        </is>
-      </c>
-      <c r="D8" s="11" t="inlineStr">
-        <is>
-          <t>62.470.324/0001-40</t>
-        </is>
-      </c>
-      <c r="E8" s="6" t="inlineStr">
-        <is>
-          <t>Pago</t>
-        </is>
-      </c>
-      <c r="F8" s="12" t="n">
-        <v>300258637</v>
-      </c>
-      <c r="G8" s="10" t="inlineStr">
-        <is>
-          <t>02/06/2026</t>
-        </is>
-      </c>
-      <c r="H8" s="13" t="inlineStr">
-        <is>
-          <t>M K INDUSTRIA TEXTIL LTDA</t>
-        </is>
-      </c>
-      <c r="I8" s="10" t="n">
-        <v>19</v>
-      </c>
-      <c r="J8" s="13" t="inlineStr">
-        <is>
-          <t>ESGARÇANDO</t>
-        </is>
-      </c>
-      <c r="K8" s="10" t="n">
-        <v>798</v>
-      </c>
-      <c r="L8" s="10" t="n">
-        <v>211.47</v>
-      </c>
-      <c r="M8" s="14" t="n">
-        <v>247.4199</v>
-      </c>
-    </row>
-    <row r="9" ht="22" customHeight="1">
-      <c r="A9" s="15" t="inlineStr">
-        <is>
-          <t>TOTAL HISTÓRICO</t>
-        </is>
-      </c>
-      <c r="M9" s="16" t="n">
-        <v>499.4613000000001</v>
-      </c>
-    </row>
-    <row r="11" ht="28" customHeight="1">
-      <c r="A11" s="17" t="inlineStr">
+    <row r="7" ht="28" customHeight="1">
+      <c r="A7" s="6" t="inlineStr">
         <is>
           <t>Documento gerado automaticamente pelo sistema de Controle de Qualidade. Este histórico acumula todas as cobranças confirmadas no período.</t>
         </is>
@@ -940,10 +630,10 @@
     </row>
   </sheetData>
   <mergeCells count="4">
-    <mergeCell ref="A2:M2"/>
-    <mergeCell ref="A11:M11"/>
-    <mergeCell ref="A9:L9"/>
-    <mergeCell ref="A1:M1"/>
+    <mergeCell ref="A7:N7"/>
+    <mergeCell ref="A2:N2"/>
+    <mergeCell ref="A5:M5"/>
+    <mergeCell ref="A1:N1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>